<commit_message>
Add PiN by pop, step 1 hybrid  for Somalia___SOM
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Somalia___SOM/PiN_pop_step1_Somalia___SOM_1022_12PM.xlsx
+++ b/platform_PiN_output/Somalia___SOM/PiN_pop_step1_Somalia___SOM_1022_12PM.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IDP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="host" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IDP" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,6 +426,1692 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>admin_2</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Population group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TotN</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>% severity levels 1-2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t># severity levels 1-2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>% severity level 3</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t># severity level 3</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>% severity level 4</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t># severity level 4</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>% severity level 5</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t># severity level 5</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>% Tot PiN (severity levels 3-5)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t># Tot PiN (severity levels 3-5)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Area severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SO1103</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>17071</v>
+      </c>
+      <c r="D2" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6973</v>
+      </c>
+      <c r="F2" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>9137</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>721</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K2" t="n">
+        <v>240</v>
+      </c>
+      <c r="L2" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="M2" t="n">
+        <v>10098</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SO1104</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>15492</v>
+      </c>
+      <c r="D3" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5850</v>
+      </c>
+      <c r="F3" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>8558</v>
+      </c>
+      <c r="H3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1083</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="M3" t="n">
+        <v>9642</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SO1202</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>36044</v>
+      </c>
+      <c r="D4" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>29828</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5652</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>440</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K4" t="n">
+        <v>126</v>
+      </c>
+      <c r="L4" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>6217</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SO1304</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>23365</v>
+      </c>
+      <c r="D5" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>10027</v>
+      </c>
+      <c r="F5" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>11039</v>
+      </c>
+      <c r="H5" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2300</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>13339</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SO1501</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>31394</v>
+      </c>
+      <c r="D6" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>13128</v>
+      </c>
+      <c r="F6" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>17368</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>652</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K6" t="n">
+        <v>245</v>
+      </c>
+      <c r="L6" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="M6" t="n">
+        <v>18265</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SO1503</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>32784</v>
+      </c>
+      <c r="D7" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8323</v>
+      </c>
+      <c r="F7" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="G7" t="n">
+        <v>23951</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="I7" t="n">
+        <v>510</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="M7" t="n">
+        <v>24461</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SO1604</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>9184</v>
+      </c>
+      <c r="D8" t="n">
+        <v>44</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4039</v>
+      </c>
+      <c r="F8" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4426</v>
+      </c>
+      <c r="H8" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="I8" t="n">
+        <v>719</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>56</v>
+      </c>
+      <c r="M8" t="n">
+        <v>5145</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SO1701</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>61170</v>
+      </c>
+      <c r="D9" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>32867</v>
+      </c>
+      <c r="F9" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>27694</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>609</v>
+      </c>
+      <c r="L9" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="M9" t="n">
+        <v>28303</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SO1801</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>182675</v>
+      </c>
+      <c r="D10" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="E10" t="n">
+        <v>92474</v>
+      </c>
+      <c r="F10" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>75041</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6064</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>9096</v>
+      </c>
+      <c r="L10" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="M10" t="n">
+        <v>90200</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SO1802</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>35703</v>
+      </c>
+      <c r="D11" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="E11" t="n">
+        <v>25213</v>
+      </c>
+      <c r="F11" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10138</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>353</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="M11" t="n">
+        <v>10491</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SO1803</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>46864</v>
+      </c>
+      <c r="D12" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>16540</v>
+      </c>
+      <c r="F12" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="G12" t="n">
+        <v>29497</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="I12" t="n">
+        <v>827</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="M12" t="n">
+        <v>30324</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SO1901</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>64063</v>
+      </c>
+      <c r="D13" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>16160</v>
+      </c>
+      <c r="F13" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>38476</v>
+      </c>
+      <c r="H13" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="I13" t="n">
+        <v>9427</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>74.8</v>
+      </c>
+      <c r="M13" t="n">
+        <v>47903</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SO1902</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>50364</v>
+      </c>
+      <c r="D14" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>23054</v>
+      </c>
+      <c r="F14" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="G14" t="n">
+        <v>26069</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1064</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K14" t="n">
+        <v>177</v>
+      </c>
+      <c r="L14" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="M14" t="n">
+        <v>27310</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SO1903</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>34105</v>
+      </c>
+      <c r="D15" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="E15" t="n">
+        <v>12231</v>
+      </c>
+      <c r="F15" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="G15" t="n">
+        <v>21247</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I15" t="n">
+        <v>157</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K15" t="n">
+        <v>470</v>
+      </c>
+      <c r="L15" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="M15" t="n">
+        <v>21874</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SO2001</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>48711</v>
+      </c>
+      <c r="D16" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>17207</v>
+      </c>
+      <c r="F16" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>30492</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="I16" t="n">
+        <v>886</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K16" t="n">
+        <v>127</v>
+      </c>
+      <c r="L16" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="M16" t="n">
+        <v>31504</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SO2002</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>11508</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E17" t="n">
+        <v>479</v>
+      </c>
+      <c r="F17" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>9590</v>
+      </c>
+      <c r="H17" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1225</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="K17" t="n">
+        <v>213</v>
+      </c>
+      <c r="L17" t="n">
+        <v>95.8</v>
+      </c>
+      <c r="M17" t="n">
+        <v>11028</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SO2003</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10539</v>
+      </c>
+      <c r="D18" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4885</v>
+      </c>
+      <c r="F18" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="G18" t="n">
+        <v>5444</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I18" t="n">
+        <v>209</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="M18" t="n">
+        <v>5653</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SO2101</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>33529</v>
+      </c>
+      <c r="D19" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1732</v>
+      </c>
+      <c r="F19" t="n">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="G19" t="n">
+        <v>29694</v>
+      </c>
+      <c r="H19" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1608</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>495</v>
+      </c>
+      <c r="L19" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="M19" t="n">
+        <v>31797</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SO2203</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>247922</v>
+      </c>
+      <c r="D20" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="E20" t="n">
+        <v>77895</v>
+      </c>
+      <c r="F20" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="G20" t="n">
+        <v>169190</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I20" t="n">
+        <v>838</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="M20" t="n">
+        <v>170028</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SO2210</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>171981</v>
+      </c>
+      <c r="D21" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="E21" t="n">
+        <v>61588</v>
+      </c>
+      <c r="F21" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="G21" t="n">
+        <v>102840</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6391</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1162</v>
+      </c>
+      <c r="L21" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="M21" t="n">
+        <v>110393</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SO2301</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>60213</v>
+      </c>
+      <c r="D22" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>36775</v>
+      </c>
+      <c r="F22" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G22" t="n">
+        <v>23056</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I22" t="n">
+        <v>191</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K22" t="n">
+        <v>191</v>
+      </c>
+      <c r="L22" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="M22" t="n">
+        <v>23437</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SO2302</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>67918</v>
+      </c>
+      <c r="D23" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>10252</v>
+      </c>
+      <c r="F23" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>56064</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I23" t="n">
+        <v>320</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1281</v>
+      </c>
+      <c r="L23" t="n">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="M23" t="n">
+        <v>57666</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SO2401</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>156304</v>
+      </c>
+      <c r="D24" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>58056</v>
+      </c>
+      <c r="F24" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="G24" t="n">
+        <v>90433</v>
+      </c>
+      <c r="H24" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5582</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2233</v>
+      </c>
+      <c r="L24" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="M24" t="n">
+        <v>98248</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SO2402</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>38531</v>
+      </c>
+      <c r="D25" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="E25" t="n">
+        <v>10588</v>
+      </c>
+      <c r="F25" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="G25" t="n">
+        <v>24887</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I25" t="n">
+        <v>655</v>
+      </c>
+      <c r="J25" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="K25" t="n">
+        <v>2401</v>
+      </c>
+      <c r="L25" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="M25" t="n">
+        <v>27943</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SO2403</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>26900</v>
+      </c>
+      <c r="D26" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1440</v>
+      </c>
+      <c r="F26" t="n">
+        <v>89.59999999999999</v>
+      </c>
+      <c r="G26" t="n">
+        <v>24096</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I26" t="n">
+        <v>76</v>
+      </c>
+      <c r="J26" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1288</v>
+      </c>
+      <c r="L26" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="M26" t="n">
+        <v>25460</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SO2404</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>24608</v>
+      </c>
+      <c r="D27" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>13648</v>
+      </c>
+      <c r="F27" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="G27" t="n">
+        <v>9900</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="I27" t="n">
+        <v>354</v>
+      </c>
+      <c r="J27" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="K27" t="n">
+        <v>707</v>
+      </c>
+      <c r="L27" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="M27" t="n">
+        <v>10961</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SO2504</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>14254</v>
+      </c>
+      <c r="D28" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="E28" t="n">
+        <v>7948</v>
+      </c>
+      <c r="F28" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="G28" t="n">
+        <v>6306</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="M28" t="n">
+        <v>6306</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SO2602</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>26103</v>
+      </c>
+      <c r="D29" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>11078</v>
+      </c>
+      <c r="F29" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="G29" t="n">
+        <v>13879</v>
+      </c>
+      <c r="H29" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="I29" t="n">
+        <v>637</v>
+      </c>
+      <c r="J29" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" t="n">
+        <v>509</v>
+      </c>
+      <c r="L29" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="M29" t="n">
+        <v>15025</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SO2603</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>4845</v>
+      </c>
+      <c r="D30" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="E30" t="n">
+        <v>869</v>
+      </c>
+      <c r="F30" t="n">
+        <v>71</v>
+      </c>
+      <c r="G30" t="n">
+        <v>3440</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="I30" t="n">
+        <v>129</v>
+      </c>
+      <c r="J30" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="K30" t="n">
+        <v>407</v>
+      </c>
+      <c r="L30" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="M30" t="n">
+        <v>3976</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SO2604</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>9533</v>
+      </c>
+      <c r="D31" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E31" t="n">
+        <v>901</v>
+      </c>
+      <c r="F31" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="G31" t="n">
+        <v>7304</v>
+      </c>
+      <c r="H31" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1186</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K31" t="n">
+        <v>142</v>
+      </c>
+      <c r="L31" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="M31" t="n">
+        <v>8632</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SO2605</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>30168</v>
+      </c>
+      <c r="D32" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="E32" t="n">
+        <v>13749</v>
+      </c>
+      <c r="F32" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>10880</v>
+      </c>
+      <c r="H32" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="I32" t="n">
+        <v>4748</v>
+      </c>
+      <c r="J32" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="K32" t="n">
+        <v>791</v>
+      </c>
+      <c r="L32" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="M32" t="n">
+        <v>16420</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SO2606</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>5019</v>
+      </c>
+      <c r="D33" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2134</v>
+      </c>
+      <c r="F33" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2697</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I33" t="n">
+        <v>174</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K33" t="n">
+        <v>13</v>
+      </c>
+      <c r="L33" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="M33" t="n">
+        <v>2885</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>